<commit_message>
Fix workbook formula errors: replace hard-coded values in C-PESPreservation and C-RiskModel with traceable references to input and calculation sheets, resolving the Path B internal conflict and aligning attrition/amortization formulas with the Omnibus methodology
</commit_message>
<xml_diff>
--- a/FY28/RSU5_FY28_Projection.xlsx
+++ b/FY28/RSU5_FY28_Projection.xlsx
@@ -744,8 +744,9 @@
           <t>PES cost per student (from analysis)</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
-        <v>24247</v>
+      <c r="B10" s="5">
+        <f>'C-CostPremium'!B12</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -754,8 +755,9 @@
           <t>District avg cost per student</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
-        <v>15600</v>
+      <c r="B11" s="5">
+        <f>'C-CostPremium'!F12</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -764,8 +766,9 @@
           <t>PES cost premium (fixed-cost dilution)</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n">
-        <v>8647</v>
+      <c r="B12" s="7">
+        <f>'C-CostPremium'!G12</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -819,11 +822,13 @@
           <t>MS consolidation (7-8 at FMS)</t>
         </is>
       </c>
-      <c r="B20" s="7" t="n">
-        <v>154000</v>
-      </c>
-      <c r="C20" s="7" t="n">
-        <v>154000</v>
+      <c r="B20" s="7">
+        <f>'C-MSConsol'!B21</f>
+        <v/>
+      </c>
+      <c r="C20" s="7">
+        <f>'C-MSConsol'!B21</f>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -832,11 +837,13 @@
           <t>Additional efficiencies (shared services, scheduling)</t>
         </is>
       </c>
-      <c r="B21" s="10" t="n">
-        <v>325000</v>
-      </c>
-      <c r="C21" s="10" t="n">
-        <v>650000</v>
+      <c r="B21" s="10">
+        <f>'I-Assumptions'!B22</f>
+        <v/>
+      </c>
+      <c r="C21" s="10">
+        <f>'I-Assumptions'!B23</f>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -895,77 +902,72 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>PES staff savings (positions eliminated)</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="n">
-        <v>538500</v>
+          <t>True efficiency savings (marginal teacher + admin + support - coord.)</t>
+        </is>
+      </c>
+      <c r="B29" s="7">
+        <f>'C-FY28Paths'!B33</f>
+        <v/>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>~5 FTE net reduction</t>
+          <t>C-FY28Paths: 2.05 FTE teacher + Art 7 admin + 50% Art 5 - DCS coord.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Additional bus routes (Pownal -&gt; DCS)</t>
-        </is>
-      </c>
-      <c r="B30" s="73" t="n">
-        <v>-225000</v>
+          <t>All transport costs (Pownal-&gt;DCS, Freeport PreK-&gt;PES, Durham PreK-&gt;PES)</t>
+        </is>
+      </c>
+      <c r="B30" s="73">
+        <f>'C-FY28Paths'!B34</f>
+        <v/>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>3 routes @ $75,000/ea</t>
+          <t>C-FY28Paths: 3+3+2 = 8 routes at I-Assumptions cost/route</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>PES building conversion (PreK center)</t>
-        </is>
-      </c>
-      <c r="B31" s="73" t="n">
-        <v>-74375</v>
+          <t>PES EC conversion (amortized per I-Assumptions)</t>
+        </is>
+      </c>
+      <c r="B31" s="73">
+        <f>'C-FY28Paths'!B35</f>
+        <v/>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>$743,750 over 10 yrs</t>
+          <t>C-FY28Paths: I-Assumptions partial x multiplier / years</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>DCS capacity/coordination costs</t>
+          <t>(DCS coordination already included in true efficiency above)</t>
         </is>
       </c>
       <c r="B32" s="73" t="n">
-        <v>-75000</v>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>Additional admin, space prep</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>EC program opt-out risk (families choosing private)</t>
+          <t>(EC opt-out risk modeled in C-RiskModel, not direct cost)</t>
         </is>
       </c>
       <c r="B33" s="73" t="n">
-        <v>-50000</v>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>Transport barrier reduces enrollment</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
@@ -981,7 +983,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Path B net: approximately -$161K/year COST (not savings).</t>
+          <t>Path B true net: cost of ~$161K/year (from C-FY28Paths true efficiency lens).</t>
         </is>
       </c>
     </row>
@@ -1155,8 +1157,9 @@
           <t>CDS EC transfer revenue</t>
         </is>
       </c>
-      <c r="B51" s="7" t="n">
-        <v>300000</v>
+      <c r="B51" s="7">
+        <f>AVERAGE('I-ECCosts'!B29,'I-ECCosts'!C29)</f>
+        <v/>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
@@ -1170,8 +1173,9 @@
           <t>IDEA Part B federal SpEd funding</t>
         </is>
       </c>
-      <c r="B52" s="7" t="n">
-        <v>125000</v>
+      <c r="B52" s="7">
+        <f>AVERAGE('I-ECCosts'!B30,'I-ECCosts'!C30)</f>
+        <v/>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
@@ -1185,8 +1189,9 @@
           <t>EPS PreK state allocation</t>
         </is>
       </c>
-      <c r="B53" s="7" t="n">
-        <v>75000</v>
+      <c r="B53" s="7">
+        <f>AVERAGE('I-ECCosts'!B31,'I-ECCosts'!C31)</f>
+        <v/>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
@@ -1305,11 +1310,12 @@
         <v>80</v>
       </c>
       <c r="B65" s="16">
-        <f>B29*2/80</f>
-        <v/>
-      </c>
-      <c r="C65" s="7" t="n">
-        <v>12361</v>
+        <f>'C-Budget'!D7/A65</f>
+        <v/>
+      </c>
+      <c r="C65" s="7">
+        <f>B65-'C-CostPremium'!F12</f>
+        <v/>
       </c>
       <c r="D65" s="16">
         <f>B22/80</f>
@@ -1321,11 +1327,12 @@
         <v>90</v>
       </c>
       <c r="B66" s="16">
-        <f>B29*2/90</f>
-        <v/>
-      </c>
-      <c r="C66" s="7" t="n">
-        <v>10875</v>
+        <f>'C-Budget'!D7/A66</f>
+        <v/>
+      </c>
+      <c r="C66" s="7">
+        <f>B66-'C-CostPremium'!F12</f>
+        <v/>
       </c>
       <c r="D66" s="16">
         <f>B22/90</f>
@@ -1337,11 +1344,12 @@
         <v>100</v>
       </c>
       <c r="B67" s="16">
-        <f>B29*2/100</f>
-        <v/>
-      </c>
-      <c r="C67" s="7" t="n">
-        <v>9389</v>
+        <f>'C-Budget'!D7/A67</f>
+        <v/>
+      </c>
+      <c r="C67" s="7">
+        <f>B67-'C-CostPremium'!F12</f>
+        <v/>
       </c>
       <c r="D67" s="16">
         <f>B22/100</f>
@@ -1353,11 +1361,12 @@
         <v>105</v>
       </c>
       <c r="B68" s="16">
-        <f>B29*2/105</f>
-        <v/>
-      </c>
-      <c r="C68" s="7" t="n">
-        <v>8647</v>
+        <f>'C-Budget'!D7/A68</f>
+        <v/>
+      </c>
+      <c r="C68" s="7">
+        <f>B68-'C-CostPremium'!F12</f>
+        <v/>
       </c>
       <c r="D68" s="16">
         <f>B22/105</f>
@@ -1369,11 +1378,12 @@
         <v>110</v>
       </c>
       <c r="B69" s="16">
-        <f>B29*2/110</f>
-        <v/>
-      </c>
-      <c r="C69" s="7" t="n">
-        <v>7904</v>
+        <f>'C-Budget'!D7/A69</f>
+        <v/>
+      </c>
+      <c r="C69" s="7">
+        <f>B69-'C-CostPremium'!F12</f>
+        <v/>
       </c>
       <c r="D69" s="16">
         <f>B22/110</f>
@@ -1385,11 +1395,12 @@
         <v>120</v>
       </c>
       <c r="B70" s="16">
-        <f>B29*2/120</f>
-        <v/>
-      </c>
-      <c r="C70" s="7" t="n">
-        <v>6418</v>
+        <f>'C-Budget'!D7/A70</f>
+        <v/>
+      </c>
+      <c r="C70" s="7">
+        <f>B70-'C-CostPremium'!F12</f>
+        <v/>
       </c>
       <c r="D70" s="16">
         <f>B22/120</f>
@@ -1401,11 +1412,12 @@
         <v>130</v>
       </c>
       <c r="B71" s="16">
-        <f>B29*2/130</f>
-        <v/>
-      </c>
-      <c r="C71" s="7" t="n">
-        <v>4932</v>
+        <f>'C-Budget'!D7/A71</f>
+        <v/>
+      </c>
+      <c r="C71" s="7">
+        <f>B71-'C-CostPremium'!F12</f>
+        <v/>
       </c>
       <c r="D71" s="16">
         <f>B22/130</f>
@@ -10847,22 +10859,22 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Pownal state aid (FY25-26)</t>
+          <t>Pownal total state aid (FY27)</t>
         </is>
       </c>
       <c r="B28" s="7">
-        <f>'I-Tax'!E41</f>
+        <f>'I-Revenue'!B11</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>State aid per PES student</t>
+          <t>State aid per Pownal student (all grades)</t>
         </is>
       </c>
       <c r="B29" s="7">
-        <f>B28/B27</f>
+        <f>B28/'I-Equity'!B24</f>
         <v/>
       </c>
     </row>
@@ -10952,7 +10964,7 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>At 10% attrition: 10-11 students leave, ~$50K/yr in state revenue lost to RSU 5.</t>
+          <t>At 10% attrition: ~11 students leave, ~$30K/yr in state revenue lost to RSU 5.</t>
         </is>
       </c>
     </row>
@@ -11407,19 +11419,19 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>One-time costs (amortized 5 years)</t>
+          <t>One-time costs (amortized per I-Assumptions)</t>
         </is>
       </c>
       <c r="B75" s="7">
-        <f>B63/5</f>
+        <f>B63/'I-Assumptions'!B19</f>
         <v/>
       </c>
       <c r="C75" s="7">
-        <f>AVERAGE(B63,C63)/5</f>
+        <f>AVERAGE(B63,C63)/'I-Assumptions'!B19</f>
         <v/>
       </c>
       <c r="D75" s="7">
-        <f>C63/5</f>
+        <f>C63/'I-Assumptions'!B19</f>
         <v/>
       </c>
     </row>

</xml_diff>